<commit_message>
docs(competitor-intel): add 'Tech / models' column to the dataset + fix two rows
- New column recording the AI models each competitor runs on, filled
  where disclosed (MeltFlex: GPT+Gemini 2.5 Flash Image+Veo+Seedance;
  REimagine: SD inpainting; Homestyler: NVIDIA Edify) — rest '—'.
- Fix unquoted-comma rows (Decorilla, Modsy) that had truncated the
  'What it is' cell in the previous xlsx.
- Regenerate spreadsheet; add a 'How to read' note for the new column.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GMthZ7e9Ci2vBGcvDENBzx
</commit_message>
<xml_diff>
--- a/docs/competitor-intel/DesignatureStudio-Competitors-2026-Q3.xlsx
+++ b/docs/competitor-intel/DesignatureStudio-Competitors-2026-Q3.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to read" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitors Q3 2026'!$A$1:$K$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitors Q3 2026'!$A$1:$L$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -542,6 +542,7 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
     <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -601,6 +602,12 @@
           <t>Does NOT cover / Gaps</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Tech / models
+(where known)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -658,6 +665,11 @@
           <t>No human designer; no AR; automated matching; EUR/EU-centric</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI GPT + Google Gemini 2.5 Flash Image ('Nano Banana') + Veo + Seedance (video). Orchestration layer, no proprietary model (founder-disclosed, Aug 2026).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -715,6 +727,11 @@
           <t>No human, no floor plans, no quiz; pricier tiers</t>
         </is>
       </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -772,6 +789,11 @@
           <t>No human designer (AI + chat only); automated matching not curated; real-estate skew; no quiz; no local AM market</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Stable Diffusion inpainting w/ automatic (editable) masking; architecture-preserving.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -811,22 +833,27 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Premium human-led online design</t>
+          <t>Premium human-led online design, two competing designer concepts, AI+VR assist; launched Spain Sept 2025 (Europe push)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> two competing designer concepts</t>
+          <t>From ~$299; full-room ~$539–$1,499/room; hourly $119–$500</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AI+VR assist; launched Spain Sept 2025 (Europe push)</t>
+          <t>2 designers' concepts, custom 3D + floor plan + palette, shopping list w/ up to 45% trade discount + ordering concierge, worldwide remote</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>From ~$299; full-room ~$539–$1,499/room; hourly $119–$500</t>
+          <t>No free/low self-serve AI tier; expensive entry; slow/high-touch; no local AM/RU language</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -886,6 +913,11 @@
           <t>No true $19/$49 micro-tiers; steers to house brands; renders weaker than old Modsy</t>
         </is>
       </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -943,6 +975,11 @@
           <t>No floor plans, no human, no quiz; shopping = match not curated PDF</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1000,6 +1037,11 @@
           <t>No human designer, no add-all-to-cart depth, no AR, no quiz</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1057,6 +1099,11 @@
           <t>No floor plans, no human, no quiz; furniture = suggestions not curated PDF</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1114,6 +1161,11 @@
           <t>No free AI tier; no instant AI; no AR; pricier per room</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1171,6 +1223,11 @@
           <t>No human; no quiz; gamified/grindy UX; hobbyist quality; app-only</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1228,6 +1285,11 @@
           <t>No generative AI photo redesign; no in-house human designers; shopping via trade not instant checkout</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1285,6 +1347,11 @@
           <t>No shoppable list, no floor plans, no human, no quiz, no AR</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1342,6 +1409,11 @@
           <t>IKEA catalog only (retailer-locked); no multi-retailer list; no independent advice; no paid human service</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1399,6 +1471,11 @@
           <t>Wayfair catalog only; no human; no quiz; no subscription/service tier</t>
         </is>
       </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1456,6 +1533,11 @@
           <t>No shoppable links, no floor plans, no quiz; realtor skew; few styles</t>
         </is>
       </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1513,6 +1595,11 @@
           <t>No AI self-serve; no 3D; solo capacity; small-space niche</t>
         </is>
       </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1570,6 +1657,11 @@
           <t>No signs of active operation; likely dormant</t>
         </is>
       </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1627,6 +1719,11 @@
           <t>Very expensive/aspirational; consult-only, not managed packages; no free tier</t>
         </is>
       </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1684,6 +1781,11 @@
           <t>Limited generative AI; human = referral not in-app consult; no single AI shoppable list</t>
         </is>
       </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1741,6 +1843,11 @@
           <t>B2B for designers not homeowners; no consumer photo redesign; sourcing not consumer checkout; no in-house team</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1798,6 +1905,11 @@
           <t>DIY-first; no photo-to-AI redesign; human styling is peripheral add-on; brand catalog not open checkout</t>
         </is>
       </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1855,6 +1967,11 @@
           <t>DIY tool; no human designers; no curated shoppable checkout; no quiz</t>
         </is>
       </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>AI Designer on NVIDIA Edify + AI floor planner / 'Home Copilot'.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1912,6 +2029,11 @@
           <t>You do the design; no human designer; no shoppable checkout to retailers; no consult</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1969,6 +2091,11 @@
           <t>Renders NOT shoppable (no buy links); no human; no quiz; credit caps; B2B/staging lean</t>
         </is>
       </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2026,6 +2153,11 @@
           <t>No human, no true shoppable list, no quiz, no AR</t>
         </is>
       </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2083,6 +2215,11 @@
           <t>No shoppable links, no floor plans, no human, no quiz</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2140,6 +2277,11 @@
           <t>No shoppable, no floor plans, no human, no quiz</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2197,6 +2339,11 @@
           <t>No shopping list, no floor plans, no human, no quiz; expensive</t>
         </is>
       </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2254,6 +2401,11 @@
           <t>No shoppable, no floor plans, no human, no quiz; opaque pricing</t>
         </is>
       </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2311,6 +2463,11 @@
           <t>No shoppable, no floor plans, no human, no quiz; thin feature set</t>
         </is>
       </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2368,6 +2525,11 @@
           <t>No shopping list, no floor plans, no human, no quiz, minimal editing</t>
         </is>
       </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2425,6 +2587,11 @@
           <t>No shoppable links, no floor plans, no human, no quiz; credit model</t>
         </is>
       </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2482,6 +2649,11 @@
           <t>No remote worldwide; no AI self-serve tiers; no Armenian market</t>
         </is>
       </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2539,6 +2711,11 @@
           <t>No worldwide remote-only; no low-cost AI self-serve; no Armenian market; capital-heavy</t>
         </is>
       </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2596,6 +2773,11 @@
           <t>No AI photo redesign headline; no human; no shoppable; no consult</t>
         </is>
       </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2653,6 +2835,11 @@
           <t>No AI photo redesign; no productized remote tiers; no style quiz; no shoppable lists; no worldwide self-serve</t>
         </is>
       </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2710,6 +2897,11 @@
           <t>No shoppable matching; no retailer catalog; no AR; no AI-instant; sells to agents</t>
         </is>
       </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2767,6 +2959,11 @@
           <t>No shoppable products; no retailer catalog; no AR; light on floor plans</t>
         </is>
       </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2824,6 +3021,11 @@
           <t>No shoppable products (that lives in REimagineHome); no AR; agent-focused</t>
         </is>
       </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2881,6 +3083,11 @@
           <t>No currently-marketed shoppable buy-list/AR self-serve; realtor/enterprise focus</t>
         </is>
       </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2938,6 +3145,11 @@
           <t>Outdoor only; no free AI; pricey; revisions extra</t>
         </is>
       </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2995,6 +3207,11 @@
           <t>No human; predatory weekly-sub funnel; name-confusion clones; model placement not direct shop links; variable quality</t>
         </is>
       </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3052,6 +3269,11 @@
           <t>No human; no shoppable list; no quiz; no AR; thin; clone listings</t>
         </is>
       </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3109,6 +3331,11 @@
           <t>No human; no curated shoppable list; no quiz; staging-first; inconsistent pricing</t>
         </is>
       </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3166,6 +3393,11 @@
           <t>Builder/remodeler pros; limited AI; no consumer redesign/shopping/human</t>
         </is>
       </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3223,6 +3455,11 @@
           <t>Credit model; pro positioning; no human service; no consumer cart</t>
         </is>
       </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3280,6 +3517,11 @@
           <t>Pro-oriented; no 1-click photo redesign; no human service; no consumer shopping; learning curve</t>
         </is>
       </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3337,6 +3579,11 @@
           <t>Manual DIY; essentially no generative AI; no human; no shopping service</t>
         </is>
       </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3394,6 +3641,11 @@
           <t>Floor-plan/layout focus not styled rooms; no photo redesign; no shopping; no human</t>
         </is>
       </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3451,6 +3703,11 @@
           <t>iOS/Mac only; no 3D/floor plans; no render; no human; no direct checkout</t>
         </is>
       </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3508,6 +3765,11 @@
           <t>Designer B2B; no consumer photo redesign; no DTC shopping; no in-house designers</t>
         </is>
       </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3565,6 +3827,11 @@
           <t>Back-office studio tool; no AI room gen; no rendering focus; no consumer service</t>
         </is>
       </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3622,6 +3889,11 @@
           <t>Floor-plan-centric; minimal AI; no photo restyle; no ecommerce; no full styling</t>
         </is>
       </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3679,6 +3951,11 @@
           <t>No shopping, no real floor plans (misleading name), no human/quiz/account; low control</t>
         </is>
       </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3736,6 +4013,11 @@
           <t>No shoppable links, no floor plans, no human, no quiz; no real free tier</t>
         </is>
       </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3793,6 +4075,11 @@
           <t>No shopping, no floor plans, no human, no quiz; pro/arch</t>
         </is>
       </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3850,6 +4137,11 @@
           <t>No shoppable, no floor plan gen, no human, no quiz; CAD workflow</t>
         </is>
       </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3907,6 +4199,11 @@
           <t>No shopping, no floor plans, no human, no quiz; clone-tier</t>
         </is>
       </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3964,6 +4261,11 @@
           <t>No remote worldwide; no AI photo tools headline; no low-cost tiers</t>
         </is>
       </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4021,6 +4323,11 @@
           <t>No human; no shoppable; no floor plans; no quiz; no consult</t>
         </is>
       </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4078,6 +4385,11 @@
           <t>No productized remote self-serve; no low-cost tiers; no Armenian/CIS market</t>
         </is>
       </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4135,6 +4447,11 @@
           <t>No human; no shoppable buy-list; no floor plans; no quiz; staging tool</t>
         </is>
       </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4192,6 +4509,11 @@
           <t>No generative AI redesign; no styles/guidance; no human; Amazon catalog only</t>
         </is>
       </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4249,6 +4571,11 @@
           <t>No photo redesign; no AR-in-space; no human; no quiz; inspiration + shopping not design gen</t>
         </is>
       </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4306,6 +4633,11 @@
           <t>No full-room furnishing; no AI concept gen; no human; flooring/surfaces only</t>
         </is>
       </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4363,6 +4695,11 @@
           <t>Bassett product-bound; no AI; some studios closing</t>
         </is>
       </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4420,6 +4757,11 @@
           <t>CB2 product only; no AI self-serve</t>
         </is>
       </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4477,6 +4819,11 @@
           <t>C&amp;B catalog-bound; no AI self-serve</t>
         </is>
       </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4534,6 +4881,11 @@
           <t>Ethan Allen product-centric; no AI; higher-end</t>
         </is>
       </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4591,6 +4943,11 @@
           <t>PB/Williams-Sonoma catalog; Room Planner is config not generative AI</t>
         </is>
       </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4648,6 +5005,11 @@
           <t>R&amp;B product only; no AI; no free self-serve tool</t>
         </is>
       </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4705,6 +5067,11 @@
           <t>West Elm catalog only; no AI self-serve; no independent list</t>
         </is>
       </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4762,6 +5129,11 @@
           <t>No shoppable products; no retailer catalog; no human</t>
         </is>
       </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4819,6 +5191,11 @@
           <t>No shoppable products; no retailer catalog; no AR; agent workflow</t>
         </is>
       </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4876,6 +5253,11 @@
           <t>No shoppable matching, no retailer catalog, no AR, no human, no floor plans</t>
         </is>
       </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4933,6 +5315,11 @@
           <t>Not an e-design competitor; furniture brand in Havenly ecosystem</t>
         </is>
       </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4990,6 +5377,11 @@
           <t>B2B pro sampling not room design; no redesign/shopping-for-consumers</t>
         </is>
       </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5047,6 +5439,11 @@
           <t>No room-accurate photo redesign; no human; no shoppable; no floor plans; no quiz</t>
         </is>
       </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5104,6 +5501,11 @@
           <t>No room-accurate redesign; no human; no shoppable; no floor plans; no quiz</t>
         </is>
       </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5161,6 +5563,11 @@
           <t>No room-accurate redesign; no human; no shoppable; no floor plans; no quiz</t>
         </is>
       </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5218,6 +5625,11 @@
           <t>No AI redesign; no human; no shop links; no quiz; manual modeling; dated</t>
         </is>
       </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5275,6 +5687,11 @@
           <t>Not a decorating tool; no AI redesign/styles/shopping; contractor field tool</t>
         </is>
       </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5332,6 +5749,11 @@
           <t>Kitchen/bath niche; dealer/pro only; no whole-home AI; no consumer service</t>
         </is>
       </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5389,6 +5811,11 @@
           <t>Infra/API for developers; no consumer UI; no styling/redesign/shopping</t>
         </is>
       </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5446,6 +5873,11 @@
           <t>Steep learning curve; pro pricing; minimal AI; no redesign/shopping/human</t>
         </is>
       </c>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5503,6 +5935,11 @@
           <t>Architect early-design niche; no interiors styling; no consumer render/shopping</t>
         </is>
       </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5560,6 +5997,11 @@
           <t>Enterprise procurement niche; no rendering/redesign/consumer; no styling service</t>
         </is>
       </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5617,6 +6059,11 @@
           <t>B2B — not a consumer purchase; no consumer AI self-serve</t>
         </is>
       </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5674,6 +6121,11 @@
           <t>Visualization only; bring your own model; no authoring/AI/service/shopping</t>
         </is>
       </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5731,6 +6183,11 @@
           <t>Steep learning curve; model everything yourself; no photo redesign; no shopping/human</t>
         </is>
       </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5788,6 +6245,11 @@
           <t>Developer feasibility not interiors; no room render; no consumer anything</t>
         </is>
       </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5845,6 +6307,11 @@
           <t>DEAD — collapsed with parent Bed Bath &amp; Beyond</t>
         </is>
       </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -5902,6 +6369,11 @@
           <t>DEAD — never built operational infrastructure</t>
         </is>
       </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5959,6 +6431,11 @@
           <t>Interior app wound down; team pivoted (gaming); precedent that standalone shoppable-room app is hard</t>
         </is>
       </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6016,6 +6493,11 @@
           <t>DEAD — marketing overspend + quality problems</t>
         </is>
       </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6055,27 +6537,32 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Original AI/3D-render + human designer</t>
+          <t>Original AI/3D-render + human designer, shoppable — the archetype of Designature's model</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> shoppable — the archetype of Designature's model</t>
+          <t>(historic) ~$69–$159/room</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>(historic) ~$69–$159/room</t>
+          <t>3D renders, human designer, shoppable list</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>3D renders, human designer, shoppable list</t>
+          <t>DEAD — died on render costs / human-design margins. Cautionary tale</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K97"/>
+  <autoFilter ref="A1:L97"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -6182,7 +6669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6316,22 +6803,38 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
+          <t>Tech / models column</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>AI models each tool runs on, filled only where publicly disclosed or founder-confirmed (most are '—' — a research field to fill over quarters). Key insight: MeltFlex uses off-the-shelf GPT + Gemini 2.5 Flash Image + Veo/Seedance = no model moat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr"/>
+      <c r="B16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
           <t>Refresh cadence</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Quarterly. Re-run the same 6-segment scan; compare vs prior quarter's CSV in git history.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Source of truth CSV</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>docs/competitor-intel/competitors-2026-Q3.csv</t>
         </is>

</xml_diff>